<commit_message>
Update A2700 source test configuration
</commit_message>
<xml_diff>
--- a/config/A2700/Source_Test_A2700M.xlsx
+++ b/config/A2700/Source_Test_A2700M.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PNT\61.AI\VisionOCR\config\A2700\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76D37C8-8A63-4664-A50E-1D8E233EFEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699A6D21-5560-43A6-AB13-568C2C9373D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4455" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4593" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4585" uniqueCount="633">
   <si>
     <t>TC_ID</t>
   </si>
@@ -1930,6 +1930,26 @@
   </si>
   <si>
     <t>=0.5 ÷ Expected × 100</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A27_SPEC-TC0003-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HOME &gt; VOLTAGE &gt; Fundamental</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>65, 150</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>65,185</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>198 ~ 202; 198 ~ 202; 198 ~ 202; 198 ~ 202</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1937,6 +1957,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1977,7 +2000,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1985,6 +2008,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -6260,7 +6284,7 @@
         <v>225</v>
       </c>
       <c r="G127">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H127">
         <v>1</v>
@@ -6286,7 +6310,7 @@
         <v>225</v>
       </c>
       <c r="G129">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H129">
         <v>1</v>
@@ -19163,8 +19187,8 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>16</v>
+      <c r="A8" s="2" t="s">
+        <v>628</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -19386,14 +19410,14 @@
       <c r="E24" t="s">
         <v>427</v>
       </c>
-      <c r="F24" t="s">
-        <v>430</v>
+      <c r="F24" s="5" t="s">
+        <v>631</v>
       </c>
       <c r="H24">
         <v>0.5</v>
       </c>
-      <c r="I24" t="s">
-        <v>431</v>
+      <c r="I24" s="2" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
@@ -19412,14 +19436,14 @@
       <c r="E26" t="s">
         <v>427</v>
       </c>
-      <c r="F26" t="s">
-        <v>428</v>
+      <c r="F26" s="5" t="s">
+        <v>631</v>
       </c>
       <c r="H26">
         <v>0.5</v>
       </c>
-      <c r="I26" t="s">
-        <v>429</v>
+      <c r="I26" s="2" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.45">
@@ -19438,8 +19462,8 @@
       <c r="E28" t="s">
         <v>427</v>
       </c>
-      <c r="F28" t="s">
-        <v>430</v>
+      <c r="F28" s="2" t="s">
+        <v>630</v>
       </c>
       <c r="H28">
         <v>0.5</v>
@@ -20543,6 +20567,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -21926,8 +21951,8 @@
       <c r="C79" t="s">
         <v>473</v>
       </c>
-      <c r="H79" t="s">
-        <v>484</v>
+      <c r="H79" s="1" t="s">
+        <v>528</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.45">
@@ -22022,20 +22047,6 @@
         <v>482</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A84" t="s">
-        <v>40</v>
-      </c>
-      <c r="B84" t="s">
-        <v>288</v>
-      </c>
-      <c r="C84" t="s">
-        <v>483</v>
-      </c>
-      <c r="H84" t="s">
-        <v>483</v>
-      </c>
-    </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>44</v>
@@ -22046,8 +22057,8 @@
       <c r="C86" t="s">
         <v>473</v>
       </c>
-      <c r="H86" t="s">
-        <v>474</v>
+      <c r="H86" s="1" t="s">
+        <v>528</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.45">
@@ -22142,20 +22153,6 @@
         <v>482</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
-        <v>44</v>
-      </c>
-      <c r="B91" t="s">
-        <v>289</v>
-      </c>
-      <c r="C91" t="s">
-        <v>483</v>
-      </c>
-      <c r="H91" t="s">
-        <v>483</v>
-      </c>
-    </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>56</v>
@@ -22307,7 +22304,7 @@
         <v>320</v>
       </c>
       <c r="F101">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H101" t="s">
         <v>337</v>
@@ -22330,7 +22327,7 @@
         <v>320</v>
       </c>
       <c r="F102">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H102" t="s">
         <v>487</v>
@@ -22353,7 +22350,7 @@
         <v>320</v>
       </c>
       <c r="F103">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H103" t="s">
         <v>489</v>
@@ -22376,7 +22373,7 @@
         <v>320</v>
       </c>
       <c r="F104">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H104" t="s">
         <v>482</v>
@@ -23509,8 +23506,8 @@
       <c r="I169" t="s">
         <v>492</v>
       </c>
-      <c r="J169" t="s">
-        <v>607</v>
+      <c r="J169" s="2" t="s">
+        <v>632</v>
       </c>
       <c r="L169" t="s">
         <v>391</v>

</xml_diff>